<commit_message>
Data: only sourced values, no stand-ins
- Mars targets: exact sourced coordinates (Jezero landing site, Arcadia AP-1) with a
  coordinate source each; drop the planet-wide temperature used as a site value.
- Earth sites on a lake or the sea: slope and relief marked not measured instead of
  using the water surface (neutral in the score).
- About: hide the challenge name and Use of AI until filled in, instead of placeholder text.
</commit_message>
<xml_diff>
--- a/analysis/mars-among-us-analog-data.xlsx
+++ b/analysis/mars-among-us-analog-data.xlsx
@@ -1723,12 +1723,8 @@
       <c r="N11" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="O11" s="13" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>25</v>
-      </c>
+      <c r="O11" s="13" t="n"/>
+      <c r="P11" s="10" t="n"/>
       <c r="Q11" s="10" t="inlineStr">
         <is>
           <t>Ice-cored permafrost mounds</t>
@@ -1737,7 +1733,7 @@
       <c r="R11" s="12" t="n"/>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>DEM: DEM samples at sea level/water near the coast: slope unreliable.</t>
+          <t>DEM: Coordinates fall on water near the coast: slope and relief not measured.</t>
         </is>
       </c>
       <c r="T11" s="10" t="inlineStr">
@@ -2183,12 +2179,8 @@
       <c r="N17" s="10" t="n">
         <v>477</v>
       </c>
-      <c r="O17" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="O17" s="13" t="n"/>
+      <c r="P17" s="10" t="n"/>
       <c r="Q17" s="10" t="inlineStr">
         <is>
           <t>Basalt (impact crater)</t>
@@ -2197,7 +2189,7 @@
       <c r="R17" s="12" t="n"/>
       <c r="S17" s="10" t="inlineStr">
         <is>
-          <t>DEM: Coordinates fall on the crater lake surface: slope reflects the lake, not the crater walls.</t>
+          <t>DEM: Coordinates fall on the crater lake: slope and relief not measured.</t>
         </is>
       </c>
       <c r="T17" s="10" t="inlineStr">
@@ -2651,12 +2643,8 @@
       <c r="N23" s="10" t="n">
         <v>326</v>
       </c>
-      <c r="O23" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P23" s="10" t="n">
-        <v>8</v>
-      </c>
+      <c r="O23" s="13" t="n"/>
+      <c r="P23" s="10" t="n"/>
       <c r="Q23" s="10" t="inlineStr">
         <is>
           <t>Anorthosite, granodiorite, mangerite; impact melt</t>
@@ -2665,7 +2653,7 @@
       <c r="R23" s="12" t="n"/>
       <c r="S23" s="10" t="inlineStr">
         <is>
-          <t>Analog for lunar highland craters. Rock types: craterexplorer.ca. Coordinates: approximate area centre. DEM: Coordinates fall on Mistastin Lake: slope reflects the lake surface.</t>
+          <t>Analog for lunar highland craters. Rock types: craterexplorer.ca. Coordinates: approximate area centre. DEM: Coordinates fall on Mistastin Lake: slope and relief not measured.</t>
         </is>
       </c>
       <c r="T23" s="10" t="inlineStr">
@@ -3581,10 +3569,10 @@
         </is>
       </c>
       <c r="F37" s="11" t="n">
-        <v>18</v>
+        <v>18.44</v>
       </c>
       <c r="G37" s="11" t="n">
-        <v>77</v>
+        <v>77.45</v>
       </c>
       <c r="H37" s="12" t="n"/>
       <c r="I37" s="14" t="n"/>
@@ -3599,12 +3587,12 @@
       <c r="R37" s="12" t="n"/>
       <c r="S37" s="10" t="inlineStr">
         <is>
-          <t>Perseverance landing site. Approximate: JPL press kit gives "about 18° latitude, 77° longitude".</t>
+          <t>Perseverance landing site (Octavia E. Butler Landing), 18.44° N, 77.45° E.</t>
         </is>
       </c>
       <c r="T37" s="10" t="inlineStr">
         <is>
-          <t>https://www.jpl.nasa.gov/news/press_kits/mars_2020/launch/mission/landing_site/</t>
+          <t>https://en.wikipedia.org/wiki/Octavia_E._Butler_Landing</t>
         </is>
       </c>
       <c r="U37" s="12" t="n"/>
@@ -3785,10 +3773,10 @@
         </is>
       </c>
       <c r="F41" s="11" t="n">
-        <v>40</v>
+        <v>39.8</v>
       </c>
       <c r="G41" s="11" t="n">
-        <v>-162</v>
+        <v>-157.9</v>
       </c>
       <c r="H41" s="12" t="n"/>
       <c r="I41" s="14" t="n"/>
@@ -3803,7 +3791,7 @@
       <c r="R41" s="12" t="n"/>
       <c r="S41" s="10" t="inlineStr">
         <is>
-          <t>Ice-rich candidate landing region; centre of the published box 37–43° N, 192–204° E.</t>
+          <t>Candidate human landing site AP-1 (39.8° N, 202.1° E), with evidence of near-surface ice (Luzzi et al. 2025).</t>
         </is>
       </c>
       <c r="T41" s="10" t="inlineStr">
@@ -4189,7 +4177,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>See each row. Jezero is approximate (about 18° N, 77° E).</t>
+          <t>See each row.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mars targets: add sourced day-night swing and slope
- Gale: day-night swing about 70 °C (REMS, NASA/JPL PIA16913).
- Jezero: 61 °C on one sample day (MEDA, NASA/JPL first weather report).
- Oxia Planum: landing ellipse avoids slopes above 8° at the MOLA sub-kilometre scale.
- Score the day-night swing (3 within 10 °C, 2 within 30 °C, else 1).
- Rover landing slope limits over 2-5 m are not used: not comparable with the 300 m Earth slopes.
  Victoria, Arcadia and Mars relief have no comparable published value yet.
</commit_message>
<xml_diff>
--- a/analysis/mars-among-us-analog-data.xlsx
+++ b/analysis/mars-among-us-analog-data.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="اقرأني" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purposes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sites" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; method" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini review" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="اقرأني" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Purposes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sites" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sources &amp; method" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gemini review" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sites'!$A$1:$U$51</definedName>
@@ -3576,7 +3576,9 @@
       </c>
       <c r="H37" s="12" t="n"/>
       <c r="I37" s="14" t="n"/>
-      <c r="J37" s="14" t="n"/>
+      <c r="J37" s="14" t="n">
+        <v>61</v>
+      </c>
       <c r="K37" s="12" t="n"/>
       <c r="L37" s="12" t="n"/>
       <c r="M37" s="12" t="n"/>
@@ -3587,7 +3589,7 @@
       <c r="R37" s="12" t="n"/>
       <c r="S37" s="10" t="inlineStr">
         <is>
-          <t>Perseverance landing site (Octavia E. Butler Landing), 18.44° N, 77.45° E.</t>
+          <t>Perseverance landing site (Octavia E. Butler Landing), 18.44° N, 77.45° E. Day–night swing: one sample day (sols 43–44), high −22 °C, low −83 °C (MEDA; NASA/JPL, https://www.jpl.nasa.gov/news/nasas-first-weather-report-from-jezero-crater-on-mars/).</t>
         </is>
       </c>
       <c r="T37" s="10" t="inlineStr">
@@ -3627,7 +3629,9 @@
       </c>
       <c r="H38" s="12" t="n"/>
       <c r="I38" s="14" t="n"/>
-      <c r="J38" s="14" t="n"/>
+      <c r="J38" s="14" t="n">
+        <v>70</v>
+      </c>
       <c r="K38" s="12" t="n"/>
       <c r="L38" s="12" t="n"/>
       <c r="M38" s="12" t="n"/>
@@ -3638,7 +3642,7 @@
       <c r="R38" s="12" t="n"/>
       <c r="S38" s="10" t="inlineStr">
         <is>
-          <t>Curiosity landing site (Bradbury Landing).</t>
+          <t>Curiosity landing site (Bradbury Landing). Day–night swing: daily highs about 0 °C, lows about −70 °C (REMS; NASA/JPL, https://www.jpl.nasa.gov/images/pia16913-steady-temperatures-at-mars-gale-crater/).</t>
         </is>
       </c>
       <c r="T38" s="10" t="inlineStr">
@@ -3689,7 +3693,7 @@
       <c r="R39" s="12" t="n"/>
       <c r="S39" s="10" t="inlineStr">
         <is>
-          <t>ExoMars Rosalind Franklin landing site; centre of the published high-resolution map (18.20° N, 335.45° E).</t>
+          <t>ExoMars Rosalind Franklin landing site; centre of the published high-resolution map (18.20° N, 335.45° E). Landing ellipse avoids slopes &gt;8° at the MOLA sub-kilometre scale (Quantin-Nataf et al. 2021).</t>
         </is>
       </c>
       <c r="T39" s="10" t="inlineStr">

</xml_diff>